<commit_message>
Update bp alias version from 3.1.0 to 3.2.0 12ac4890f8ac40a873eadfaded1ed028a97b639b
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-MESObservationBmi.xlsx
+++ b/main/ig/StructureDefinition-MESObservationBmi.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-26T14:10:46+00:00</t>
+    <t>2026-03-12T14:12:24+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1906,7 +1906,7 @@
     <t>JDV_J148-ReferenceRangeAppliesTo-CISIS</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J148-ReferenceRangeAppliesTo-CISIS/FHIR/JDV-J148-ReferenceRangeAppliesTo-CISIS|1.2.0</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J148-ReferenceRangeAppliesTo-CISIS/FHIR/JDV-J148-ReferenceRangeAppliesTo-CISIS|20250131120000</t>
   </si>
   <si>
     <t>Observation.referenceRange.appliesTo.id</t>
@@ -2460,7 +2460,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="84.54296875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="100.9140625" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="110.9140625" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>

</xml_diff>